<commit_message>
Further added Rock-Type Mapping for Yukon, Chile, Gandaki and Hessen
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Rock-Type_Manual.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Rock-Type_Manual.xlsx
@@ -8,17 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_AD4DB114E441178AC67DF498FE16CBA4683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27F12C89-0583-4769-BBD9-B1737E05DED6}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="11_AD4DB114E441178AC67DF498FE16CBA4683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27C38768-BFB6-4722-A1CA-743365658E01}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Allgemein" sheetId="1" r:id="rId1"/>
     <sheet name="REFLECT" sheetId="3" r:id="rId2"/>
     <sheet name="MDPI Tibet" sheetId="2" r:id="rId3"/>
     <sheet name="CAES2014" sheetId="4" r:id="rId4"/>
     <sheet name="ALPS" sheetId="5" r:id="rId5"/>
     <sheet name="Yukon" sheetId="6" r:id="rId6"/>
+    <sheet name="Chile" sheetId="7" r:id="rId7"/>
+    <sheet name="Gandaki mmc1" sheetId="8" r:id="rId8"/>
+    <sheet name="Hessen" sheetId="9" r:id="rId9"/>
+    <sheet name="MDPI Xianshuie" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="118">
   <si>
     <t>USGS</t>
   </si>
@@ -255,6 +259,135 @@
   </si>
   <si>
     <t>Hinzufügen</t>
+  </si>
+  <si>
+    <t>vorher</t>
+  </si>
+  <si>
+    <t>Angepasst</t>
+  </si>
+  <si>
+    <t>Verallgemeinerung</t>
+  </si>
+  <si>
+    <t>GANDAKI mmc1</t>
+  </si>
+  <si>
+    <t>Vereinfachung</t>
+  </si>
+  <si>
+    <t>Unconsolidated rocks</t>
+  </si>
+  <si>
+    <t>Arkose, Sandstone, Conglomerate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slate, Sandstone </t>
+  </si>
+  <si>
+    <t>Slate</t>
+  </si>
+  <si>
+    <t>extra Zeile erzeugen</t>
+  </si>
+  <si>
+    <t>Gneiss, Greenschist</t>
+  </si>
+  <si>
+    <t>Pelite, Halite rock</t>
+  </si>
+  <si>
+    <t>Halite</t>
+  </si>
+  <si>
+    <t>Sandstone, Limestone, Granite</t>
+  </si>
+  <si>
+    <t>Unconsolidated rocks, Carbonate bearing silt</t>
+  </si>
+  <si>
+    <t>Phyllite</t>
+  </si>
+  <si>
+    <t>Marl</t>
+  </si>
+  <si>
+    <t>Pelite, Sandstone, Conglomerate</t>
+  </si>
+  <si>
+    <t>Graywacke, Dolerite</t>
+  </si>
+  <si>
+    <t>Dolerite</t>
+  </si>
+  <si>
+    <t>Dolomite, Pelite</t>
+  </si>
+  <si>
+    <t>Graywacke, Slate</t>
+  </si>
+  <si>
+    <t>Unconsolidated rocks, Marl</t>
+  </si>
+  <si>
+    <t>Quartzite, Slate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slate </t>
+  </si>
+  <si>
+    <t>Pelite, Sandstone</t>
+  </si>
+  <si>
+    <t>Slate, Pelite</t>
+  </si>
+  <si>
+    <t>Tuff, Hawaiite</t>
+  </si>
+  <si>
+    <t>Tuff</t>
+  </si>
+  <si>
+    <t>Muscovite-Biotite-Gneiss</t>
+  </si>
+  <si>
+    <t>Dolomite, Pelite, Limestone, Anhydrite</t>
+  </si>
+  <si>
+    <t>Marl, Pelite, Limestone</t>
+  </si>
+  <si>
+    <t>Arkose</t>
+  </si>
+  <si>
+    <t>Limestone, Arkose, Pelite</t>
+  </si>
+  <si>
+    <t>Slate, Volcanic rocks</t>
+  </si>
+  <si>
+    <t>Slate, Graywacke</t>
+  </si>
+  <si>
+    <t>Graywacke</t>
+  </si>
+  <si>
+    <t>Marl, Dolomite</t>
+  </si>
+  <si>
+    <t>Slate, Graywacke, Dolerite</t>
+  </si>
+  <si>
+    <t>Gneiss, Phyllite</t>
+  </si>
+  <si>
+    <t>MDPI Xianshuihe</t>
+  </si>
+  <si>
+    <t>voorher</t>
+  </si>
+  <si>
+    <t>Angeapasst</t>
   </si>
 </sst>
 </file>
@@ -278,7 +411,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,6 +430,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -310,13 +449,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -711,9 +851,46 @@
       <c r="B14" t="s">
         <v>25</v>
       </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A598BD8F-FFD8-45C4-A108-3D5C20239D87}">
+  <dimension ref="B3:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1020,7 +1197,7 @@
       <c r="D4" t="s">
         <v>60</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1031,7 +1208,7 @@
       <c r="D5" t="s">
         <v>61</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1042,7 +1219,7 @@
       <c r="D6" t="s">
         <v>62</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1053,7 +1230,7 @@
       <c r="D7" t="s">
         <v>63</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1064,7 +1241,7 @@
       <c r="D8" t="s">
         <v>64</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1075,7 +1252,7 @@
       <c r="D9" t="s">
         <v>65</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1086,7 +1263,7 @@
       <c r="D10" t="s">
         <v>66</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1097,7 +1274,7 @@
       <c r="D11" t="s">
         <v>67</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1108,7 +1285,7 @@
       <c r="D12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1119,7 +1296,7 @@
       <c r="D13" t="s">
         <v>69</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1130,7 +1307,7 @@
       <c r="D14" t="s">
         <v>70</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1144,15 +1321,519 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96018C36-E3E3-41C1-A1D4-74C08BA8B199}">
-  <dimension ref="B3"/>
+  <dimension ref="B3:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
         <v>25</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{046163C6-310B-4276-B13A-C4313804DA44}">
+  <dimension ref="B3:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3AA3BB1-9300-4FF4-9EB8-EFBB770A4269}">
+  <dimension ref="B3:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="16.85546875" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E633D5F-8493-4434-94EF-89F9E3029D40}">
+  <dimension ref="B3:F43"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="45.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="20.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>96</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="29" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>100</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>101</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>94</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>102</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>106</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
+        <v>107</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>108</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>109</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="39" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>98</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="40" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>110</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>113</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="43" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>114</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Special cases for rock-type mapping in USGS database and fixed Problem for rock-type mapping. should work fine now
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Rock-Type_Manual.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Rock-Type_Manual.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="97" documentId="11_AD4DB114E441178AC67DF498FE16CBA4683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCDE0A4D-5200-4C4C-BCF4-8635E2CFF9E9}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21870" yWindow="2640" windowWidth="21600" windowHeight="11295" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Allgemein" sheetId="1" r:id="rId1"/>
@@ -701,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -709,7 +709,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1203,7 +1202,7 @@
       </c>
     </row>
     <row r="4" spans="2:4">
-      <c r="C4" s="5" t="s">
+      <c r="C4" t="s">
         <v>119</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1211,7 +1210,7 @@
       </c>
     </row>
     <row r="5" spans="2:4">
-      <c r="C5" s="5" t="s">
+      <c r="C5" t="s">
         <v>120</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1269,12 +1268,12 @@
       </c>
     </row>
     <row r="3" spans="2:8">
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="4" spans="2:8">
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1282,7 +1281,7 @@
       </c>
     </row>
     <row r="5" spans="2:8">
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1290,7 +1289,7 @@
       </c>
     </row>
     <row r="6" spans="2:8">
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>121</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -1298,7 +1297,7 @@
       </c>
     </row>
     <row r="7" spans="2:8">
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -1306,7 +1305,7 @@
       </c>
     </row>
     <row r="8" spans="2:8">
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>122</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -1317,7 +1316,7 @@
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>124</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -1325,7 +1324,7 @@
       </c>
     </row>
     <row r="10" spans="2:8">
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>125</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1336,7 +1335,7 @@
       </c>
     </row>
     <row r="11" spans="2:8">
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>126</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -1344,7 +1343,7 @@
       </c>
     </row>
     <row r="12" spans="2:8">
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>127</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -1355,7 +1354,7 @@
       </c>
     </row>
     <row r="13" spans="2:8">
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1363,7 +1362,7 @@
       </c>
     </row>
     <row r="14" spans="2:8">
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>129</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1374,7 +1373,7 @@
       </c>
     </row>
     <row r="15" spans="2:8">
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -1385,7 +1384,7 @@
       </c>
     </row>
     <row r="16" spans="2:8">
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>142</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -1393,7 +1392,7 @@
       </c>
     </row>
     <row r="17" spans="3:6">
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>143</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -1404,7 +1403,7 @@
       </c>
     </row>
     <row r="18" spans="3:6">
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>144</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -1418,7 +1417,7 @@
       </c>
     </row>
     <row r="19" spans="3:6">
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>145</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -1426,7 +1425,7 @@
       </c>
     </row>
     <row r="20" spans="3:6">
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1434,7 +1433,7 @@
       </c>
     </row>
     <row r="21" spans="3:6">
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>146</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -1442,7 +1441,7 @@
       </c>
     </row>
     <row r="22" spans="3:6">
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>147</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -1450,7 +1449,7 @@
       </c>
     </row>
     <row r="23" spans="3:6">
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>148</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1461,7 +1460,7 @@
       </c>
     </row>
     <row r="24" spans="3:6">
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>149</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -1475,7 +1474,7 @@
       </c>
     </row>
     <row r="25" spans="3:6">
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>150</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1483,7 +1482,7 @@
       </c>
     </row>
     <row r="26" spans="3:6">
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>151</v>
       </c>
       <c r="D26" s="1" t="s">
@@ -1494,7 +1493,7 @@
       </c>
     </row>
     <row r="27" spans="3:6">
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>161</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -1508,7 +1507,7 @@
       </c>
     </row>
     <row r="28" spans="3:6">
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>163</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -1522,7 +1521,7 @@
       </c>
     </row>
     <row r="29" spans="3:6">
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>164</v>
       </c>
       <c r="D29" s="1" t="s">
@@ -1536,7 +1535,7 @@
       </c>
     </row>
     <row r="30" spans="3:6">
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>165</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -1547,7 +1546,7 @@
       </c>
     </row>
     <row r="31" spans="3:6">
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>166</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -1555,7 +1554,7 @@
       </c>
     </row>
     <row r="32" spans="3:6">
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>167</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -1566,7 +1565,7 @@
       </c>
     </row>
     <row r="33" spans="3:7">
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="5" t="s">
         <v>168</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1574,7 +1573,7 @@
       </c>
     </row>
     <row r="34" spans="3:7">
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="5" t="s">
         <v>169</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -1588,7 +1587,7 @@
       </c>
     </row>
     <row r="35" spans="3:7">
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="5" t="s">
         <v>170</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1605,7 +1604,7 @@
       </c>
     </row>
     <row r="36" spans="3:7">
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="5" t="s">
         <v>171</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -1616,7 +1615,7 @@
       </c>
     </row>
     <row r="37" spans="3:7">
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>172</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -1624,7 +1623,7 @@
       </c>
     </row>
     <row r="38" spans="3:7">
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="5" t="s">
         <v>173</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -1638,7 +1637,7 @@
       </c>
     </row>
     <row r="39" spans="3:7">
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="5" t="s">
         <v>174</v>
       </c>
       <c r="D39" s="1" t="s">
@@ -1649,7 +1648,7 @@
       </c>
     </row>
     <row r="40" spans="3:7">
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="5" t="s">
         <v>175</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -1663,7 +1662,7 @@
       </c>
     </row>
     <row r="41" spans="3:7">
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>176</v>
       </c>
       <c r="D41" s="1" t="s">
@@ -1671,7 +1670,7 @@
       </c>
     </row>
     <row r="42" spans="3:7">
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="5" t="s">
         <v>177</v>
       </c>
       <c r="D42" s="1" t="s">
@@ -1685,7 +1684,7 @@
       </c>
     </row>
     <row r="43" spans="3:7">
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="5" t="s">
         <v>178</v>
       </c>
       <c r="D43" s="1" t="s">
@@ -1696,7 +1695,7 @@
       </c>
     </row>
     <row r="44" spans="3:7">
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="5" t="s">
         <v>179</v>
       </c>
       <c r="D44" s="1" t="s">
@@ -1707,7 +1706,7 @@
       </c>
     </row>
     <row r="45" spans="3:7">
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="5" t="s">
         <v>180</v>
       </c>
       <c r="D45" s="1" t="s">
@@ -1715,7 +1714,7 @@
       </c>
     </row>
     <row r="46" spans="3:7">
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="5" t="s">
         <v>181</v>
       </c>
       <c r="D46" s="1" t="s">
@@ -1726,7 +1725,7 @@
       </c>
     </row>
     <row r="47" spans="3:7">
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="5" t="s">
         <v>182</v>
       </c>
       <c r="D47" s="1" t="s">
@@ -1740,7 +1739,7 @@
       </c>
     </row>
     <row r="48" spans="3:7">
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="5" t="s">
         <v>183</v>
       </c>
       <c r="D48" s="1" t="s">
@@ -1754,7 +1753,7 @@
       </c>
     </row>
     <row r="49" spans="3:8">
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="5" t="s">
         <v>184</v>
       </c>
       <c r="D49" s="1" t="s">
@@ -1771,7 +1770,7 @@
       </c>
     </row>
     <row r="50" spans="3:8">
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="5" t="s">
         <v>185</v>
       </c>
       <c r="D50" s="1" t="s">
@@ -1785,7 +1784,7 @@
       </c>
     </row>
     <row r="51" spans="3:8">
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="5" t="s">
         <v>186</v>
       </c>
       <c r="D51" s="1" t="s">
@@ -1796,7 +1795,7 @@
       </c>
     </row>
     <row r="52" spans="3:8">
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="5" t="s">
         <v>187</v>
       </c>
       <c r="D52" s="1" t="s">
@@ -1810,7 +1809,7 @@
       </c>
     </row>
     <row r="53" spans="3:8">
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="5" t="s">
         <v>188</v>
       </c>
       <c r="D53" s="1" t="s">
@@ -1821,7 +1820,7 @@
       </c>
     </row>
     <row r="54" spans="3:8">
-      <c r="C54" s="6" t="s">
+      <c r="C54" s="5" t="s">
         <v>189</v>
       </c>
       <c r="D54" s="1" t="s">
@@ -1835,7 +1834,7 @@
       </c>
     </row>
     <row r="55" spans="3:8">
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="5" t="s">
         <v>190</v>
       </c>
       <c r="D55" s="1" t="s">
@@ -1852,7 +1851,7 @@
       </c>
     </row>
     <row r="56" spans="3:8">
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="5" t="s">
         <v>191</v>
       </c>
       <c r="D56" s="1" t="s">
@@ -1866,7 +1865,7 @@
       </c>
     </row>
     <row r="57" spans="3:8">
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="5" t="s">
         <v>192</v>
       </c>
       <c r="D57" s="1" t="s">
@@ -1874,7 +1873,7 @@
       </c>
     </row>
     <row r="58" spans="3:8">
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="5" t="s">
         <v>193</v>
       </c>
       <c r="D58" s="1" t="s">
@@ -1891,7 +1890,7 @@
       </c>
     </row>
     <row r="59" spans="3:8">
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="5" t="s">
         <v>194</v>
       </c>
       <c r="D59" s="1" t="s">
@@ -1905,7 +1904,7 @@
       </c>
     </row>
     <row r="60" spans="3:8">
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="5" t="s">
         <v>195</v>
       </c>
       <c r="D60" s="1" t="s">
@@ -1925,7 +1924,7 @@
       </c>
     </row>
     <row r="61" spans="3:8">
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="5" t="s">
         <v>196</v>
       </c>
       <c r="D61" s="1" t="s">
@@ -1936,7 +1935,7 @@
       </c>
     </row>
     <row r="62" spans="3:8">
-      <c r="C62" s="6" t="s">
+      <c r="C62" s="5" t="s">
         <v>197</v>
       </c>
       <c r="D62" s="1" t="s">
@@ -1944,7 +1943,7 @@
       </c>
     </row>
     <row r="63" spans="3:8">
-      <c r="C63" s="6" t="s">
+      <c r="C63" s="5" t="s">
         <v>162</v>
       </c>
       <c r="D63" s="1" t="s">
@@ -1952,7 +1951,7 @@
       </c>
     </row>
     <row r="64" spans="3:8">
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="5" t="s">
         <v>160</v>
       </c>
       <c r="D64" s="1" t="s">
@@ -1963,7 +1962,7 @@
       </c>
     </row>
     <row r="65" spans="3:8">
-      <c r="C65" s="6" t="s">
+      <c r="C65" s="5" t="s">
         <v>159</v>
       </c>
       <c r="D65" s="1" t="s">
@@ -1974,7 +1973,7 @@
       </c>
     </row>
     <row r="66" spans="3:8">
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="5" t="s">
         <v>158</v>
       </c>
       <c r="D66" s="1" t="s">
@@ -1994,7 +1993,7 @@
       </c>
     </row>
     <row r="67" spans="3:8">
-      <c r="C67" s="6" t="s">
+      <c r="C67" s="5" t="s">
         <v>157</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -2005,7 +2004,7 @@
       </c>
     </row>
     <row r="68" spans="3:8">
-      <c r="C68" s="6" t="s">
+      <c r="C68" s="5" t="s">
         <v>156</v>
       </c>
       <c r="D68" s="1" t="s">
@@ -2016,7 +2015,7 @@
       </c>
     </row>
     <row r="69" spans="3:8">
-      <c r="C69" s="6" t="s">
+      <c r="C69" s="5" t="s">
         <v>155</v>
       </c>
       <c r="D69" s="1" t="s">
@@ -2027,7 +2026,7 @@
       </c>
     </row>
     <row r="70" spans="3:8">
-      <c r="C70" s="6" t="s">
+      <c r="C70" s="5" t="s">
         <v>154</v>
       </c>
       <c r="D70" s="1" t="s">
@@ -2035,7 +2034,7 @@
       </c>
     </row>
     <row r="71" spans="3:8">
-      <c r="C71" s="6" t="s">
+      <c r="C71" s="5" t="s">
         <v>153</v>
       </c>
       <c r="D71" s="1" t="s">
@@ -2046,7 +2045,7 @@
       </c>
     </row>
     <row r="72" spans="3:8">
-      <c r="C72" s="6" t="s">
+      <c r="C72" s="5" t="s">
         <v>152</v>
       </c>
       <c r="D72" s="1" t="s">
@@ -2057,7 +2056,7 @@
       </c>
     </row>
     <row r="73" spans="3:8">
-      <c r="C73" s="6" t="s">
+      <c r="C73" s="5" t="s">
         <v>140</v>
       </c>
       <c r="D73" s="1" t="s">
@@ -2068,7 +2067,7 @@
       </c>
     </row>
     <row r="74" spans="3:8">
-      <c r="C74" s="6" t="s">
+      <c r="C74" s="5" t="s">
         <v>139</v>
       </c>
       <c r="D74" s="1" t="s">
@@ -2082,7 +2081,7 @@
       </c>
     </row>
     <row r="75" spans="3:8">
-      <c r="C75" s="6" t="s">
+      <c r="C75" s="5" t="s">
         <v>138</v>
       </c>
       <c r="D75" s="1" t="s">
@@ -2102,7 +2101,7 @@
       </c>
     </row>
     <row r="76" spans="3:8">
-      <c r="C76" s="6" t="s">
+      <c r="C76" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D76" s="1" t="s">
@@ -2119,7 +2118,7 @@
       </c>
     </row>
     <row r="77" spans="3:8">
-      <c r="C77" s="6" t="s">
+      <c r="C77" s="5" t="s">
         <v>136</v>
       </c>
       <c r="D77" s="1" t="s">
@@ -2136,7 +2135,7 @@
       </c>
     </row>
     <row r="78" spans="3:8">
-      <c r="C78" s="6" t="s">
+      <c r="C78" s="5" t="s">
         <v>135</v>
       </c>
       <c r="D78" s="1" t="s">
@@ -2153,7 +2152,7 @@
       </c>
     </row>
     <row r="79" spans="3:8">
-      <c r="C79" s="6" t="s">
+      <c r="C79" s="5" t="s">
         <v>134</v>
       </c>
       <c r="D79" s="1" t="s">
@@ -2167,7 +2166,7 @@
       </c>
     </row>
     <row r="80" spans="3:8">
-      <c r="C80" s="6" t="s">
+      <c r="C80" s="5" t="s">
         <v>133</v>
       </c>
       <c r="D80" s="1" t="s">
@@ -2178,7 +2177,7 @@
       </c>
     </row>
     <row r="81" spans="3:7">
-      <c r="C81" s="6" t="s">
+      <c r="C81" s="5" t="s">
         <v>132</v>
       </c>
       <c r="D81" s="1" t="s">
@@ -2195,7 +2194,7 @@
       </c>
     </row>
     <row r="82" spans="3:7">
-      <c r="C82" s="6" t="s">
+      <c r="C82" s="5" t="s">
         <v>131</v>
       </c>
       <c r="D82" s="1" t="s">
@@ -2212,7 +2211,7 @@
       </c>
     </row>
     <row r="83" spans="3:7">
-      <c r="C83" s="6" t="s">
+      <c r="C83" s="5" t="s">
         <v>130</v>
       </c>
       <c r="D83" s="1" t="s">

</xml_diff>